<commit_message>
feat: Add bonus round functionality to quiz results and update import logic
</commit_message>
<xml_diff>
--- a/data/quizzes/20260304_Casino.xlsx
+++ b/data/quizzes/20260304_Casino.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/90d082bf22ee60bf/Sonstiges/Pub Quiz/Data/2026/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{33E97CE9-CFC7-427B-B1B8-DA7D542958E4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="4" documentId="8_{33E97CE9-CFC7-427B-B1B8-DA7D542958E4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{4A150591-BF32-4FBC-984B-9BEAA016CCDE}"/>
   <bookViews>
-    <workbookView xWindow="5100" yWindow="1730" windowWidth="28800" windowHeight="15370" xr2:uid="{5DE7F39E-DF3E-4985-A3C8-10E2CCE84CC4}"/>
+    <workbookView xWindow="38290" yWindow="-110" windowWidth="38620" windowHeight="21100" xr2:uid="{5DE7F39E-DF3E-4985-A3C8-10E2CCE84CC4}"/>
   </bookViews>
   <sheets>
     <sheet name="Tabelle1" sheetId="1" r:id="rId1"/>
@@ -1184,10 +1184,10 @@
       <c r="I13" s="8">
         <v>3</v>
       </c>
-      <c r="J13" s="9">
-        <v>6</v>
-      </c>
-      <c r="K13" s="8">
+      <c r="J13" s="8">
+        <v>6</v>
+      </c>
+      <c r="K13" s="9">
         <v>11</v>
       </c>
       <c r="L13" s="8">
@@ -1571,7 +1571,7 @@
       <c r="F22" s="8">
         <v>2</v>
       </c>
-      <c r="G22" s="8">
+      <c r="G22" s="9">
         <v>6</v>
       </c>
       <c r="H22" s="8">
@@ -1580,7 +1580,7 @@
       <c r="I22" s="8">
         <v>2</v>
       </c>
-      <c r="J22" s="9">
+      <c r="J22" s="8">
         <v>10</v>
       </c>
       <c r="K22" s="8">
@@ -1596,7 +1596,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="23" spans="1:14" ht="42" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:14" ht="28" x14ac:dyDescent="0.35">
       <c r="A23" s="12">
         <v>21</v>
       </c>
@@ -1860,7 +1860,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="29" spans="1:14" ht="42" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:14" ht="28" x14ac:dyDescent="0.35">
       <c r="A29" s="12">
         <v>28</v>
       </c>

</xml_diff>

<commit_message>
feat: Enhance event difficulty reporting and validation in quiz imports
</commit_message>
<xml_diff>
--- a/data/quizzes/20260304_Casino.xlsx
+++ b/data/quizzes/20260304_Casino.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/90d082bf22ee60bf/Sonstiges/Pub Quiz/Data/2026/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="4" documentId="8_{33E97CE9-CFC7-427B-B1B8-DA7D542958E4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{4A150591-BF32-4FBC-984B-9BEAA016CCDE}"/>
+  <xr:revisionPtr revIDLastSave="23" documentId="8_{33E97CE9-CFC7-427B-B1B8-DA7D542958E4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{1F0E6CCB-1916-495B-92FB-92EF96FECFC0}"/>
   <bookViews>
     <workbookView xWindow="38290" yWindow="-110" windowWidth="38620" windowHeight="21100" xr2:uid="{5DE7F39E-DF3E-4985-A3C8-10E2CCE84CC4}"/>
   </bookViews>
@@ -306,6 +306,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -627,6 +631,9 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D7FC7A20-2399-4B24-8F7D-32AA2B612DB7}">
   <dimension ref="A1:N31"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="2" max="2" width="28.90625" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:14" ht="28" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
@@ -716,7 +723,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="3" spans="1:14" ht="28" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A3" s="11">
         <v>2</v>
       </c>
@@ -739,13 +746,13 @@
         <v>3</v>
       </c>
       <c r="H3" s="8">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="I3" s="9">
         <v>10</v>
       </c>
       <c r="J3" s="8">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="K3" s="8">
         <v>5</v>
@@ -786,10 +793,10 @@
         <v>5</v>
       </c>
       <c r="I4" s="8">
+        <v>4</v>
+      </c>
+      <c r="J4" s="8">
         <v>9</v>
-      </c>
-      <c r="J4" s="8">
-        <v>4</v>
       </c>
       <c r="K4" s="8">
         <v>4</v>
@@ -804,7 +811,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="5" spans="1:14" ht="28" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A5" s="12">
         <v>4</v>
       </c>
@@ -830,10 +837,10 @@
         <v>5</v>
       </c>
       <c r="I5" s="8">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="J5" s="8">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="K5" s="8">
         <v>5</v>
@@ -874,10 +881,10 @@
         <v>10</v>
       </c>
       <c r="I6" s="8">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="J6" s="8">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="K6" s="8">
         <v>4</v>
@@ -892,7 +899,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="7" spans="1:14" ht="28" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A7" s="12">
         <v>6</v>
       </c>
@@ -918,10 +925,10 @@
         <v>4</v>
       </c>
       <c r="I7" s="8">
+        <v>5</v>
+      </c>
+      <c r="J7" s="8">
         <v>9</v>
-      </c>
-      <c r="J7" s="8">
-        <v>5</v>
       </c>
       <c r="K7" s="8">
         <v>5</v>
@@ -980,7 +987,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="9" spans="1:14" ht="42" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A9" s="12">
         <v>8</v>
       </c>
@@ -1006,10 +1013,10 @@
         <v>10</v>
       </c>
       <c r="I9" s="8">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="J9" s="8">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="K9" s="8">
         <v>4</v>
@@ -1068,7 +1075,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="11" spans="1:14" ht="28" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A11" s="12">
         <v>9</v>
       </c>
@@ -1091,13 +1098,13 @@
         <v>2</v>
       </c>
       <c r="H11" s="8">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="I11" s="9">
         <v>10</v>
       </c>
       <c r="J11" s="8">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="K11" s="8">
         <v>5</v>
@@ -1244,7 +1251,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="15" spans="1:14" ht="28" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A15" s="12">
         <v>14</v>
       </c>
@@ -1255,7 +1262,7 @@
         <v>8</v>
       </c>
       <c r="D15" s="8">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="E15" s="8">
         <v>3</v>
@@ -1273,7 +1280,7 @@
         <v>3</v>
       </c>
       <c r="J15" s="8">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="K15" s="8">
         <v>4</v>
@@ -1640,7 +1647,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="24" spans="1:14" ht="28" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A24" s="12">
         <v>23</v>
       </c>
@@ -1651,7 +1658,7 @@
         <v>8</v>
       </c>
       <c r="D24" s="8">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="E24" s="8">
         <v>3</v>
@@ -1669,7 +1676,7 @@
         <v>6</v>
       </c>
       <c r="J24" s="8">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="K24" s="8">
         <v>2</v>

</xml_diff>